<commit_message>
Add orifice losses, single flow calculation and pump operating point
</commit_message>
<xml_diff>
--- a/excel/Druckverlust_Vorlage.xlsx
+++ b/excel/Druckverlust_Vorlage.xlsx
@@ -10,6 +10,9 @@
     <sheet name="Eingabe" sheetId="1" r:id="rId1"/>
     <sheet name="Ergebnisse" sheetId="2" r:id="rId2"/>
     <sheet name="Armaturendatenbank" sheetId="3" r:id="rId3"/>
+    <sheet name="Lochblende" sheetId="4" r:id="rId4"/>
+    <sheet name="Pumpe" sheetId="5" r:id="rId5"/>
+    <sheet name="Betriebspunkte" sheetId="6" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="ArmaturenTypen">'Armaturendatenbank'!$A$5:$A$16</definedName>
@@ -66,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="100">
   <si>
     <t>Rohrleitungs-Systemkennlinie</t>
   </si>
@@ -134,6 +137,9 @@
     <t>bar</t>
   </si>
   <si>
+    <t>Einzelpunkt Q [m³/h]</t>
+  </si>
+  <si>
     <t>Zeta leer = aktueller Datenbankwert; Zahl = manuelle Ueberschreibung. Anzahl 0 deaktiviert die Zeile. Neue Zeilen per Schaltflaeche. Alle Standardwerte sind Naeherungswerte und auf die lokale Rohrgeschwindigkeit bezogen.</t>
   </si>
   <si>
@@ -288,6 +294,81 @@
   </si>
   <si>
     <t>Warnung</t>
+  </si>
+  <si>
+    <t>davon Blende [bar]</t>
+  </si>
+  <si>
+    <t>Lochblende | bleibender Druckverlust</t>
+  </si>
+  <si>
+    <t>Scharfkantige, duenne, konzentrische Blende. Cd ist eine Annahme; keine ISO-5167-Messauslegung. Rohr-Di und Lochdurchmesser manuell pruefen. Aktiv=0 deaktiviert die Blende.</t>
+  </si>
+  <si>
+    <t>Aktiv (0=aus, 1=ein)</t>
+  </si>
+  <si>
+    <t>Blenden-Nennweite DN</t>
+  </si>
+  <si>
+    <t>Tatsaechlicher Rohr-Di an Blende</t>
+  </si>
+  <si>
+    <t>Lochdurchmesser d</t>
+  </si>
+  <si>
+    <t>Durchflussbeiwert Cd</t>
+  </si>
+  <si>
+    <t>Anzahl gleicher Blenden</t>
+  </si>
+  <si>
+    <t>Modellbereich: 0,2 &lt;= d/Di &lt;= 0,75. Cd=0,61 ist ein illustrativer Startwert. Unter Re=10000 erscheint eine Unsicherheitswarnung. DN-Vorschlag ueber Schaltflaeche auf Eingabe uebernehmen; der tatsaechliche Di bleibt aenderbar. Bei abweichender Rohrweite sind Reduzierverluste separat zu ergaenzen.</t>
+  </si>
+  <si>
+    <t>Durchmesserverhaeltnis beta</t>
+  </si>
+  <si>
+    <t>Pumpenkennlinie und Betriebspunkt</t>
+  </si>
+  <si>
+    <t>NOCH NICHT BERECHNET</t>
+  </si>
+  <si>
+    <t>BEISPIELWERTE ersetzen: Q streng steigend, Foerderhoehe H streng fallend. 2 bis 1000 Tabellenzeilen; keine Leerzeilen. H in Metern der gefoerderten Fluessigkeit. Berechnung ueber Pumpenbetriebspunkt auf Eingabe. Keine Extrapolation ausserhalb der eingegebenen Kennlinie.</t>
+  </si>
+  <si>
+    <t>Pumpendruck in Spalte C wird beim Berechnen aus aktueller Dichte erzeugt. Nach jeder Aenderung erneut berechnen. Schnittpunkt und Verlustanteile stehen auf Betriebspunkte; das Diagramm erscheint rechts neben der Pumpentabelle.</t>
+  </si>
+  <si>
+    <t>Q [m3/h]</t>
+  </si>
+  <si>
+    <t>Foerderhoehe H [m]</t>
+  </si>
+  <si>
+    <t>Pumpendruck [bar]</t>
+  </si>
+  <si>
+    <t>System Q [m3/h]</t>
+  </si>
+  <si>
+    <t>Systemdruck [bar]</t>
+  </si>
+  <si>
+    <t>Einzelpunkt und Pumpenbetriebspunkt</t>
+  </si>
+  <si>
+    <t>Nach Aenderungen jeden gewuenschten Berechnungsmodus neu starten. Blendenanteil ist in Armaturen enthalten.</t>
+  </si>
+  <si>
+    <t>Einzelpunkt: NOCH NICHT BERECHNET</t>
+  </si>
+  <si>
+    <t>Schnittpunkt Pumpe / System</t>
+  </si>
+  <si>
+    <t>Pumpenschnittpunkt: NOCH NICHT BERECHNET</t>
   </si>
 </sst>
 </file>
@@ -351,13 +432,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE4F3FC"/>
+        <fgColor rgb="FF185469"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF185469"/>
+        <fgColor rgb="FFE4F3FC"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -380,18 +461,18 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="5">
     <dxf>
       <fill>
         <patternFill>
@@ -424,6 +505,9 @@
           <bgColor rgb="FFFFF3CC"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="0.000000"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -619,20 +703,252 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Nach Pumpenberechnung aktualisiert</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Pumpe</c:v>
+          </c:tx>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Pumpe!$A$21:$A$26</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>50</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Pumpe!$C$21:$C$26</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>System</c:v>
+          </c:tx>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Pumpe!$N$5:$N$205</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="201"/>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Pumpe!$O$5:$O$205</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="201"/>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+        </c:ser>
+        <c:axId val="50020001"/>
+        <c:axId val="50020002"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="50020001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Q [m³/h]</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50020002"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="50020002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" vert="horz"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Differenzdruck [bar]</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50020001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>12</xdr:col>
+      <xdr:col>13</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>26</xdr:col>
+      <xdr:col>27</xdr:col>
       <xdr:colOff>38100</xdr:colOff>
       <xdr:row>23</xdr:row>
       <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>171450</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -675,6 +991,18 @@
     <tableColumn id="2" name="Zeta"/>
     <tableColumn id="3" name="Bedingungen"/>
     <tableColumn id="4" name="Quelle / Datenqualitaet"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="tblPumpe" displayName="tblPumpe" ref="A20:C26" totalsRowShown="0">
+  <autoFilter ref="A20:C26"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="Q [m3/h]" dataDxfId="2"/>
+    <tableColumn id="2" name="Foerderhoehe H [m]" dataDxfId="2"/>
+    <tableColumn id="3" name="Pumpendruck [bar]" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -965,7 +1293,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="42.7109375" customWidth="1"/>
@@ -974,37 +1302,45 @@
     <col min="6" max="9" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:8">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
-    </row>
-    <row r="3" spans="1:4">
+      <c r="F2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
-    </row>
-    <row r="5" spans="1:4">
+      <c r="G3" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
       <c r="A5" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="5">
         <v>50</v>
       </c>
       <c r="C5" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:8">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -1015,7 +1351,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:8">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -1026,7 +1362,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:8">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -1037,7 +1373,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:8">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -1048,7 +1384,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:8">
       <c r="A10" t="s">
         <v>10</v>
       </c>
@@ -1059,7 +1395,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:8">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -1070,7 +1406,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:8">
       <c r="A12" t="s">
         <v>14</v>
       </c>
@@ -1081,7 +1417,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:8">
       <c r="A13" t="s">
         <v>16</v>
       </c>
@@ -1092,7 +1428,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:8">
       <c r="A14" t="s">
         <v>18</v>
       </c>
@@ -1103,18 +1439,18 @@
         <v>17</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:8">
       <c r="A15" t="s">
         <v>19</v>
       </c>
-      <c r="B15" s="3">
+      <c r="B15" s="5">
         <v>101</v>
       </c>
       <c r="C15" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:8">
       <c r="A16" t="s">
         <v>20</v>
       </c>
@@ -1127,7 +1463,7 @@
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -1141,168 +1477,172 @@
     </row>
     <row r="20" spans="1:4">
       <c r="A20" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B20" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C20" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D20" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="21" spans="1:4">
-      <c r="A21" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B21" s="3">
+      <c r="A21" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" s="5">
         <v>0</v>
       </c>
       <c r="C21" s="4"/>
       <c r="D21" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="22" spans="1:4">
-      <c r="A22" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="B22" s="3">
+      <c r="A22" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B22" s="5">
         <v>0</v>
       </c>
       <c r="C22" s="4"/>
       <c r="D22" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="23" spans="1:4">
-      <c r="A23" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="B23" s="3">
+      <c r="A23" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B23" s="5">
         <v>0</v>
       </c>
       <c r="C23" s="4"/>
       <c r="D23" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="24" spans="1:4">
-      <c r="A24" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="B24" s="3">
+      <c r="A24" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B24" s="5">
         <v>0</v>
       </c>
       <c r="C24" s="4"/>
       <c r="D24" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="25" spans="1:4">
-      <c r="A25" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="B25" s="3">
+      <c r="A25" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B25" s="5">
         <v>0</v>
       </c>
       <c r="C25" s="4"/>
       <c r="D25" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="26" spans="1:4">
-      <c r="A26" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="B26" s="3">
+      <c r="A26" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B26" s="5">
         <v>0</v>
       </c>
       <c r="C26" s="4"/>
       <c r="D26" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="27" spans="1:4">
-      <c r="A27" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="B27" s="3">
+      <c r="A27" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B27" s="5">
         <v>0</v>
       </c>
       <c r="C27" s="4"/>
       <c r="D27" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="28" spans="1:4">
-      <c r="A28" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="B28" s="3">
+      <c r="A28" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B28" s="5">
         <v>0</v>
       </c>
       <c r="C28" s="4"/>
       <c r="D28" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="29" spans="1:4">
-      <c r="A29" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="B29" s="3">
+      <c r="A29" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B29" s="5">
         <v>0</v>
       </c>
       <c r="C29" s="4"/>
       <c r="D29" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="30" spans="1:4">
-      <c r="A30" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="B30" s="3">
+      <c r="A30" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B30" s="5">
         <v>0</v>
       </c>
       <c r="C30" s="4"/>
       <c r="D30" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="31" spans="1:4">
-      <c r="A31" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="B31" s="3">
+      <c r="A31" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B31" s="5">
         <v>0</v>
       </c>
       <c r="C31" s="4"/>
       <c r="D31" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="32" spans="1:4">
-      <c r="A32" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="B32" s="3">
+      <c r="A32" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B32" s="5">
         <v>0</v>
       </c>
       <c r="C32" s="4"/>
       <c r="D32" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A2:D3"/>
+    <mergeCell ref="F2:H2"/>
     <mergeCell ref="A18:D19"/>
   </mergeCells>
-  <dataValidations count="12">
+  <dataValidations count="13">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G3">
+      <formula1>0</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B5">
       <formula1>DNWerte</formula1>
     </dataValidation>
@@ -1352,62 +1692,66 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="9" width="17.7109375" style="6" customWidth="1"/>
+    <col min="1" max="9" width="17.7109375" style="7" customWidth="1"/>
     <col min="10" max="10" width="16.7109375" customWidth="1"/>
     <col min="11" max="11" width="85.7109375" customWidth="1"/>
+    <col min="12" max="12" width="22.7109375" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
       <c r="A2" s="2" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
       <c r="A3" s="2" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="32" customHeight="1">
-      <c r="A4" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="B4" s="7" t="s">
+    </row>
+    <row r="4" spans="1:12" ht="32" customHeight="1">
+      <c r="A4" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="B4" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="C4" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="D4" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="E4" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="F4" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="G4" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="I4" s="7" t="s">
+      <c r="H4" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="J4" s="7" t="s">
+      <c r="I4" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="K4" s="7" t="s">
+      <c r="J4" s="3" t="s">
         <v>73</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -1434,12 +1778,12 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1453,36 +1797,36 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D4" t="s">
-        <v>45</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="G4" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>59</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B5">
         <v>0.9</v>
       </c>
       <c r="C5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F5">
         <v>10</v>
@@ -1493,16 +1837,16 @@
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B6">
         <v>0.4</v>
       </c>
       <c r="C6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F6">
         <v>15</v>
@@ -1513,16 +1857,16 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B7">
         <v>0.6</v>
       </c>
       <c r="C7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7" t="s">
         <v>48</v>
-      </c>
-      <c r="D7" t="s">
-        <v>47</v>
       </c>
       <c r="F7">
         <v>20</v>
@@ -1533,16 +1877,16 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B8">
         <v>1.8</v>
       </c>
       <c r="C8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D8" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F8">
         <v>25</v>
@@ -1553,16 +1897,16 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B9">
         <v>0.05</v>
       </c>
       <c r="C9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F9">
         <v>32</v>
@@ -1573,16 +1917,16 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B10">
         <v>0.15</v>
       </c>
       <c r="C10" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D10" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F10">
         <v>40</v>
@@ -1593,16 +1937,16 @@
     </row>
     <row r="11" spans="1:7">
       <c r="A11" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B11">
         <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D11" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F11">
         <v>50</v>
@@ -1613,16 +1957,16 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B12">
         <v>2</v>
       </c>
       <c r="C12" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F12">
         <v>65</v>
@@ -1633,16 +1977,16 @@
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B13">
         <v>2</v>
       </c>
       <c r="C13" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F13">
         <v>80</v>
@@ -1653,16 +1997,16 @@
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B14">
         <v>0.5</v>
       </c>
       <c r="C14" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D14" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F14">
         <v>100</v>
@@ -1673,16 +2017,16 @@
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B15">
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D15" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F15">
         <v>125</v>
@@ -1693,16 +2037,16 @@
     </row>
     <row r="16" spans="1:7">
       <c r="A16" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B16">
         <v>0</v>
       </c>
       <c r="C16" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D16" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F16">
         <v>150</v>
@@ -1769,4 +2113,466 @@
     <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="42.7109375" customWidth="1"/>
+    <col min="2" max="6" width="20.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" t="s">
+        <v>78</v>
+      </c>
+      <c r="B5" s="5">
+        <v>0</v>
+      </c>
+      <c r="C5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B6" s="5">
+        <v>50</v>
+      </c>
+      <c r="C6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" t="s">
+        <v>80</v>
+      </c>
+      <c r="B7" s="4">
+        <v>54.5</v>
+      </c>
+      <c r="C7" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" t="s">
+        <v>81</v>
+      </c>
+      <c r="B8" s="4">
+        <v>25</v>
+      </c>
+      <c r="C8" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" t="s">
+        <v>82</v>
+      </c>
+      <c r="B9" s="4">
+        <v>0.61</v>
+      </c>
+      <c r="C9" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" t="s">
+        <v>83</v>
+      </c>
+      <c r="B10" s="5">
+        <v>1</v>
+      </c>
+      <c r="C10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" s="2"/>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" t="s">
+        <v>85</v>
+      </c>
+      <c r="B17" s="7">
+        <f>IFERROR(B8/B7,"")</f>
+        <v>0.45871559633027525</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F3"/>
+    <mergeCell ref="A12:F15"/>
+  </mergeCells>
+  <dataValidations count="6">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B5">
+      <formula1>0</formula1>
+      <formula2>1</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B6">
+      <formula1>DNWerte</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B7">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B8">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B9">
+      <formula1>1e-06</formula1>
+      <formula2>0.999999</formula2>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B10">
+      <formula1>1</formula1>
+      <formula2>1000</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:O26"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="3" width="23.7109375" customWidth="1"/>
+    <col min="5" max="12" width="13.7109375" customWidth="1"/>
+    <col min="14" max="15" width="22.7109375" style="7" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15">
+      <c r="A1" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15">
+      <c r="A3" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15">
+      <c r="N4" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="O4" s="3" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15">
+      <c r="A5" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+    </row>
+    <row r="6" spans="1:15">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+    </row>
+    <row r="7" spans="1:15">
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+    </row>
+    <row r="8" spans="1:15">
+      <c r="A8" s="2"/>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+    </row>
+    <row r="10" spans="1:15">
+      <c r="A10" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+    </row>
+    <row r="11" spans="1:15">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+    </row>
+    <row r="12" spans="1:15">
+      <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20" t="s">
+        <v>90</v>
+      </c>
+      <c r="B20" t="s">
+        <v>91</v>
+      </c>
+      <c r="C20" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" s="4">
+        <v>0</v>
+      </c>
+      <c r="B21" s="4">
+        <v>40</v>
+      </c>
+      <c r="C21" s="7"/>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="A22" s="4">
+        <v>10</v>
+      </c>
+      <c r="B22" s="4">
+        <v>38</v>
+      </c>
+      <c r="C22" s="7"/>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="A23" s="4">
+        <v>20</v>
+      </c>
+      <c r="B23" s="4">
+        <v>32</v>
+      </c>
+      <c r="C23" s="7"/>
+    </row>
+    <row r="24" spans="1:3">
+      <c r="A24" s="4">
+        <v>30</v>
+      </c>
+      <c r="B24" s="4">
+        <v>23</v>
+      </c>
+      <c r="C24" s="7"/>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" s="4">
+        <v>40</v>
+      </c>
+      <c r="B25" s="4">
+        <v>12</v>
+      </c>
+      <c r="C25" s="7"/>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26" s="4">
+        <v>50</v>
+      </c>
+      <c r="B26" s="4">
+        <v>0</v>
+      </c>
+      <c r="C26" s="7"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A5:F8"/>
+    <mergeCell ref="A10:F12"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:O10"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="9" width="17.7109375" style="7" customWidth="1"/>
+    <col min="10" max="10" width="16.7109375" customWidth="1"/>
+    <col min="11" max="11" width="85.7109375" customWidth="1"/>
+    <col min="12" max="12" width="22.7109375" style="7" customWidth="1"/>
+    <col min="14" max="15" width="23.7109375" style="7" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12">
+      <c r="A1" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
+      <c r="A2" s="2" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="32" customHeight="1">
+      <c r="A4" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="A8" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="A9" s="2" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="32" customHeight="1">
+      <c r="A10" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="L10" s="3" t="s">
+        <v>75</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="J5:J11">
+    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Uebergang">
+      <formula>NOT(ISERROR(SEARCH("Uebergang",J5)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Kv valve losses and printable engineering calculation sheets
</commit_message>
<xml_diff>
--- a/excel/Druckverlust_Vorlage.xlsx
+++ b/excel/Druckverlust_Vorlage.xlsx
@@ -13,10 +13,15 @@
     <sheet name="Lochblende" sheetId="4" r:id="rId4"/>
     <sheet name="Pumpe" sheetId="5" r:id="rId5"/>
     <sheet name="Betriebspunkte" sheetId="6" r:id="rId6"/>
+    <sheet name="KvArmatur" sheetId="7" r:id="rId7"/>
+    <sheet name="Blende_Standalone" sheetId="8" r:id="rId8"/>
+    <sheet name="Systembericht" sheetId="9" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="ArmaturenTypen">'Armaturendatenbank'!$A$5:$A$16</definedName>
     <definedName name="DNWerte">'Armaturendatenbank'!$F$5:$F$22</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="7">Blende_Standalone!$A$1:$H$48</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="8">Systembericht!$A$1:$H$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -69,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="155">
   <si>
     <t>Rohrleitungs-Systemkennlinie</t>
   </si>
@@ -299,6 +304,9 @@
     <t>davon Blende [bar]</t>
   </si>
   <si>
+    <t>davon Kv [bar]</t>
+  </si>
+  <si>
     <t>Lochblende | bleibender Druckverlust</t>
   </si>
   <si>
@@ -369,6 +377,168 @@
   </si>
   <si>
     <t>Pumpenschnittpunkt: NOCH NICHT BERECHNET</t>
+  </si>
+  <si>
+    <t>Armatur mit Kv-Wert</t>
+  </si>
+  <si>
+    <t>Kv in m³/h: Wasser mit Referenzdichte 1000 kg/m³ bei 1 bar. Aktuellen Kv fuer die festgelegte Oeffnung verwenden, nicht ungeprueft Kvs.</t>
+  </si>
+  <si>
+    <t>Kv der Armatur</t>
+  </si>
+  <si>
+    <t>Anzahl gleicher Armaturen in Serie</t>
+  </si>
+  <si>
+    <t>Delta p [bar] = n (rho/1000) (Q/Kv)^2. Gilt als Naeherung fuer turbulente, nicht kavitierende Fluessigkeitsstroemung bei konstanter Oeffnung. Keine Viskositaets-, FL-, Kavitation- oder Choked-Flow-Korrektur. Herstellergrenzen pruefen. Der Anteil wird den Einzelwiderstaenden zugerechnet und in Spalte M separat ausgewiesen.</t>
+  </si>
+  <si>
+    <t>Drosselblende | Berechnungsblatt</t>
+  </si>
+  <si>
+    <t>Projekt</t>
+  </si>
+  <si>
+    <t>Dokument</t>
+  </si>
+  <si>
+    <t>Bearbeiter</t>
+  </si>
+  <si>
+    <t>Revision</t>
+  </si>
+  <si>
+    <t>EINGABEN | lokale, unabhaengige Berechnung</t>
+  </si>
+  <si>
+    <t>Nennweite DN</t>
+  </si>
+  <si>
+    <t>Tatsaechlicher Rohr-Di D</t>
+  </si>
+  <si>
+    <t>Blendendurchmesser d</t>
+  </si>
+  <si>
+    <t>Volumenstrom Q</t>
+  </si>
+  <si>
+    <t>Dichte rho</t>
+  </si>
+  <si>
+    <t>Dyn. Viskositaet mu</t>
+  </si>
+  <si>
+    <t>Di-Vorschlag</t>
+  </si>
+  <si>
+    <t>DN legt Di nicht fest. D manuell anhand Rohrnorm und Wandstaerke pruefen. Cd=0,61 ist nur ein Startwert.</t>
+  </si>
+  <si>
+    <t>Eingaben gueltig (1=ja)</t>
+  </si>
+  <si>
+    <t>Verhaeltnis beta</t>
+  </si>
+  <si>
+    <t>Rohrgeschwindigkeit v</t>
+  </si>
+  <si>
+    <t>m/s</t>
+  </si>
+  <si>
+    <t>Rohr-Reynolds-Zahl</t>
+  </si>
+  <si>
+    <t>Bleibender Verlustbeiwert zeta</t>
+  </si>
+  <si>
+    <t>Messdifferenzdruck</t>
+  </si>
+  <si>
+    <t>Bleibender Druckverlust</t>
+  </si>
+  <si>
+    <t>Geschwindigkeit im Loch</t>
+  </si>
+  <si>
+    <t>BERECHNUNGSFORMELN | SI im Rechenkern</t>
+  </si>
+  <si>
+    <t>β = d/D; A = πD²/4; v = (Q/3600)/A; Re = ρvD/μ</t>
+  </si>
+  <si>
+    <t>a = √[1 − β⁴(1 − Cd²)]</t>
+  </si>
+  <si>
+    <t>ζbleibend = [a/(Cd β²) − 1]²</t>
+  </si>
+  <si>
+    <t>ΔpMess = [(1 − β⁴)/(Cd² β⁴)] ρv²/2</t>
+  </si>
+  <si>
+    <t>Δpbleibend = ζbleibend ρv²/2; Pa → bar: /100000</t>
+  </si>
+  <si>
+    <t>D,d: mm → m (/1000); μ: mPa·s → Pa·s (/1000)</t>
+  </si>
+  <si>
+    <t>ANNAHMEN UND GRENZEN</t>
+  </si>
+  <si>
+    <t>Stationaere, einphasige inkompressible Newtonsche Fluessigkeit; konstante Stoffwerte. Duenne scharfkantige konzentrische Blende; 0,2 &lt;= d/D &lt;= 0,75; Cd konstant und vom Anwender zu bestaetigen. Messdifferenzdruck ist nicht bleibender Druckverlust. Druckrueckgewinnungsansatz im Zusammenhang mit ISO 5167-2; keine normgerechte Messstellenauslegung. Keine Pruefung von Kavitation, Flashing, Laerm, Erosion oder mechanischer Festigkeit. Temperatur ist nur dokumentiert.</t>
+  </si>
+  <si>
+    <t>Blatt ohne VBA lauffaehig: Formeln werden in Excel automatisch neu berechnet. Alle Daten und die DN-Vorschlagstabelle liegen lokal auf diesem Blatt. Fuer eine Freigabe Stoffdaten, Cd und Modellgrenzen fachlich pruefen. Ausdruck/PDF: A4 Hochformat, eine Seite.</t>
+  </si>
+  <si>
+    <t>Geprueft durch: ____________________    Datum: ______________    Freigabe: ______________</t>
+  </si>
+  <si>
+    <t>Systemkennlinie | Engineering-Bericht</t>
+  </si>
+  <si>
+    <t>Pumpe einschliessen (0/1)</t>
+  </si>
+  <si>
+    <t>NOCH NICHT BERECHNET | SystemberichtErstellen ausfuehren</t>
+  </si>
+  <si>
+    <t>Eingabestand wird beim Erstellen dokumentiert.</t>
+  </si>
+  <si>
+    <t>Betriebspunkt / Hinweise werden beim Erstellen dokumentiert.</t>
+  </si>
+  <si>
+    <t>WICHTIGSTE GLEICHUNGEN</t>
+  </si>
+  <si>
+    <t>v = (Q/3600)/(πD²/4); Re = ρvD/μ; laminar: λ = 64/Re</t>
+  </si>
+  <si>
+    <t>Colebrook: 1/√λ = −2 log10[ε/(3,7D) + 2,51/(Re√λ)]</t>
+  </si>
+  <si>
+    <t>ΔpR = λ(L/D)ρv²/2; ΔpE = Σ(nζ)ρv²/2</t>
+  </si>
+  <si>
+    <t>ΔpSystem = ΔpR + ΔpE + ρgΔh + ΔpBehaelter</t>
+  </si>
+  <si>
+    <t>Kv: Δp [bar] = n (ρ/1000) (Q/Kv)²; Blende: ζ = [√(1−β⁴(1−Cd²))/(Cdβ²)−1]²</t>
+  </si>
+  <si>
+    <t>Pumpe: ΔpP = ρgH(Q); Schnittpunkt: ΔpP − ΔpSystem = 0; Pa → bar: /100000</t>
+  </si>
+  <si>
+    <t>Stationaer, inkompressibel, einphasig, Newtonsch; konstante Stoffwerte. Hauptrohr mit einheitlichem D. Re=2300–4000 unsicher (Maximum aus laminar/Colebrook). Zeta/Cd/Kv angenaehert, Herstellergrenzen pruefen. Kv: konstante Oeffnung, turbulent, nicht kavitierend. Pumpen-H streng fallend, linear interpoliert, keine Extrapolation. Keine NPSH-, Phasen- oder Festigkeitspruefung. Details und Eingabestand im Anhang.</t>
+  </si>
+  <si>
+    <t>Geprueft durch: ____________________  Datum: _____________  Freigabe: ______________</t>
+  </si>
+  <si>
+    <t>ANHANG | vollstaendiger Berechnungsstand</t>
   </si>
 </sst>
 </file>
@@ -379,7 +549,7 @@
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.000000"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -411,13 +581,42 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="17"/>
+      <color rgb="FF185469"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF185469"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Cambria"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="8"/>
       <color indexed="81"/>
       <name val="Tahoma"/>
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -442,8 +641,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEDF3F5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -451,11 +656,35 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -468,6 +697,22 @@
     <xf numFmtId="1" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1692,31 +1937,31 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="9" width="17.7109375" style="7" customWidth="1"/>
     <col min="10" max="10" width="16.7109375" customWidth="1"/>
     <col min="11" max="11" width="85.7109375" customWidth="1"/>
-    <col min="12" max="12" width="22.7109375" style="7" customWidth="1"/>
+    <col min="12" max="13" width="22.7109375" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:12">
+    <row r="2" spans="1:13">
       <c r="A2" s="2" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:12">
+    <row r="3" spans="1:13">
       <c r="A3" s="2" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="32" customHeight="1">
+    <row r="4" spans="1:13" ht="32" customHeight="1">
       <c r="A4" s="3" t="s">
         <v>64</v>
       </c>
@@ -1752,6 +1997,9 @@
       </c>
       <c r="L4" s="3" t="s">
         <v>75</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -2126,12 +2374,12 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2149,7 +2397,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B5" s="5">
         <v>0</v>
@@ -2160,7 +2408,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B6" s="5">
         <v>50</v>
@@ -2171,7 +2419,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B7" s="4">
         <v>54.5</v>
@@ -2182,7 +2430,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B8" s="4">
         <v>25</v>
@@ -2193,7 +2441,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B9" s="4">
         <v>0.61</v>
@@ -2204,7 +2452,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B10" s="5">
         <v>1</v>
@@ -2215,7 +2463,7 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -2249,7 +2497,7 @@
     </row>
     <row r="17" spans="1:2">
       <c r="A17" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B17" s="7">
         <f>IFERROR(B8/B7,"")</f>
@@ -2300,25 +2548,25 @@
   <sheetData>
     <row r="1" spans="1:15">
       <c r="A1" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:15">
       <c r="A3" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4" spans="1:15">
       <c r="N4" s="3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="5" spans="1:15">
       <c r="A5" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -2352,7 +2600,7 @@
     </row>
     <row r="10" spans="1:15">
       <c r="A10" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -2378,13 +2626,13 @@
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B20" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C20" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -2462,26 +2710,26 @@
     <col min="1" max="9" width="17.7109375" style="7" customWidth="1"/>
     <col min="10" max="10" width="16.7109375" customWidth="1"/>
     <col min="11" max="11" width="85.7109375" customWidth="1"/>
-    <col min="12" max="12" width="22.7109375" style="7" customWidth="1"/>
+    <col min="12" max="13" width="22.7109375" style="7" customWidth="1"/>
     <col min="14" max="15" width="23.7109375" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
       <c r="A2" s="2" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
       <c r="A3" s="2" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" ht="32" customHeight="1">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="32" customHeight="1">
       <c r="A4" s="3" t="s">
         <v>64</v>
       </c>
@@ -2518,18 +2766,21 @@
       <c r="L4" s="3" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="8" spans="1:12">
+      <c r="M4" s="3" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
       <c r="A8" s="1" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
       <c r="A9" s="2" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" ht="32" customHeight="1">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" ht="32" customHeight="1">
       <c r="A10" s="3" t="s">
         <v>64</v>
       </c>
@@ -2565,6 +2816,9 @@
       </c>
       <c r="L10" s="3" t="s">
         <v>75</v>
+      </c>
+      <c r="M10" s="3" t="s">
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -2575,4 +2829,1212 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F13"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="42.7109375" customWidth="1"/>
+    <col min="2" max="3" width="20.7109375" customWidth="1"/>
+    <col min="4" max="6" width="18.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B5" s="4">
+        <v>0</v>
+      </c>
+      <c r="C5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" t="s">
+        <v>103</v>
+      </c>
+      <c r="B6" s="4">
+        <v>10</v>
+      </c>
+      <c r="C6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" t="s">
+        <v>104</v>
+      </c>
+      <c r="B7" s="4">
+        <v>1</v>
+      </c>
+      <c r="C7" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" s="2"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F3"/>
+    <mergeCell ref="A10:F13"/>
+  </mergeCells>
+  <dataValidations count="3">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B5">
+      <formula1>0</formula1>
+      <formula2>1</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B6">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B7">
+      <formula1>1</formula1>
+      <formula2>1000</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:N48"/>
+  <sheetFormatPr defaultRowHeight="16" customHeight="1"/>
+  <cols>
+    <col min="1" max="8" width="11.7109375" customWidth="1"/>
+    <col min="13" max="14" width="14.7109375" hidden="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" ht="16" customHeight="1">
+      <c r="A1" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+    </row>
+    <row r="2" spans="1:14" ht="16" customHeight="1">
+      <c r="A2" s="8"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
+    </row>
+    <row r="3" spans="1:14" ht="16" customHeight="1">
+      <c r="A3" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="F3" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
+    </row>
+    <row r="4" spans="1:14" ht="16" customHeight="1">
+      <c r="A4" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="B4" s="10"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="F4" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="G4" s="10"/>
+      <c r="H4" s="10"/>
+    </row>
+    <row r="5" spans="1:14" ht="16" customHeight="1">
+      <c r="M5">
+        <v>10</v>
+      </c>
+      <c r="N5">
+        <v>13.6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" ht="16" customHeight="1">
+      <c r="A6" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="B6" s="11"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="11"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+      <c r="M6">
+        <v>15</v>
+      </c>
+      <c r="N6">
+        <v>17.3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="16" customHeight="1">
+      <c r="M7">
+        <v>20</v>
+      </c>
+      <c r="N7">
+        <v>22.3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" ht="16" customHeight="1">
+      <c r="A8" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="12">
+        <v>50</v>
+      </c>
+      <c r="E8" s="12"/>
+      <c r="F8" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="H8" s="9"/>
+      <c r="M8">
+        <v>25</v>
+      </c>
+      <c r="N8">
+        <v>28.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" ht="16" customHeight="1">
+      <c r="A9" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="B9" s="9"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="12">
+        <v>54.5</v>
+      </c>
+      <c r="E9" s="12"/>
+      <c r="F9" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="G9" s="13">
+        <f>IFERROR(VLOOKUP(D8,$M$5:$N$22,2,FALSE),NA())</f>
+        <v>54.5</v>
+      </c>
+      <c r="H9" s="13"/>
+      <c r="M9">
+        <v>32</v>
+      </c>
+      <c r="N9">
+        <v>37.2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" ht="16" customHeight="1">
+      <c r="A10" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="B10" s="9"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="12">
+        <v>25</v>
+      </c>
+      <c r="E10" s="12"/>
+      <c r="F10" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="G10" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="H10" s="14"/>
+      <c r="M10">
+        <v>40</v>
+      </c>
+      <c r="N10">
+        <v>43.1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" ht="16" customHeight="1">
+      <c r="A11" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="B11" s="9"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="12">
+        <v>10</v>
+      </c>
+      <c r="E11" s="12"/>
+      <c r="F11" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="G11" s="14"/>
+      <c r="H11" s="14"/>
+      <c r="M11">
+        <v>50</v>
+      </c>
+      <c r="N11">
+        <v>54.5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="16" customHeight="1">
+      <c r="A12" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="12">
+        <v>998.2</v>
+      </c>
+      <c r="E12" s="12"/>
+      <c r="F12" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="G12" s="14"/>
+      <c r="H12" s="14"/>
+      <c r="M12">
+        <v>65</v>
+      </c>
+      <c r="N12">
+        <v>70.3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" ht="16" customHeight="1">
+      <c r="A13" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="12">
+        <v>1.002</v>
+      </c>
+      <c r="E13" s="12"/>
+      <c r="F13" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G13" s="14"/>
+      <c r="H13" s="14"/>
+      <c r="M13">
+        <v>80</v>
+      </c>
+      <c r="N13">
+        <v>82.5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="16" customHeight="1">
+      <c r="A14" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="12">
+        <v>0.61</v>
+      </c>
+      <c r="E14" s="12"/>
+      <c r="F14" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="G14" s="14"/>
+      <c r="H14" s="14"/>
+      <c r="M14">
+        <v>100</v>
+      </c>
+      <c r="N14">
+        <v>107.1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" ht="16" customHeight="1">
+      <c r="A15" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="12">
+        <v>20</v>
+      </c>
+      <c r="E15" s="12"/>
+      <c r="F15" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="G15" s="14"/>
+      <c r="H15" s="14"/>
+      <c r="M15">
+        <v>125</v>
+      </c>
+      <c r="N15">
+        <v>131.7</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" ht="16" customHeight="1">
+      <c r="M16">
+        <v>150</v>
+      </c>
+      <c r="N16">
+        <v>159.3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" ht="16" customHeight="1">
+      <c r="A17" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="13">
+        <f>IFERROR(IF(AND(COUNTIF($M$5:$M$22,D8)=1,D9&gt;0,D10&gt;0,D11&gt;=0,D12&gt;0,D13&gt;0,D14&gt;0,D14&lt;1,D10/D9&gt;=0.2-1E-12,D10/D9&lt;=0.75+1E-12,OR(ISBLANK(D15),AND(ISNUMBER(D15),D15&gt;=-273.15)),ISNUMBER(D8),ISNUMBER(D9),ISNUMBER(D10),ISNUMBER(D11),ISNUMBER(D12),ISNUMBER(D13),ISNUMBER(D14)),1,0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="E17" s="13"/>
+      <c r="M17">
+        <v>200</v>
+      </c>
+      <c r="N17">
+        <v>210.1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" ht="16" customHeight="1">
+      <c r="A18" s="14" t="str">
+        <f>IF(D17&lt;&gt;1,"UNGUELTIG: Eingaben pruefen; Ergebnisse nicht verwendbar.",IF(AND(D11&gt;0,D22&lt;10000),"WARNUNG: Re &lt; 10000, konstantes Cd besonders unsicher.","Modellannahmen pruefen; keine Kavitationserkennung, keine ISO-5167-Konformitaet."))</f>
+        <v>Beim Oeffnen in Excel neu berechnen.</v>
+      </c>
+      <c r="B18" s="14"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="14"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="14"/>
+      <c r="H18" s="14"/>
+      <c r="M18">
+        <v>250</v>
+      </c>
+      <c r="N18">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" ht="16" customHeight="1">
+      <c r="A19" s="14"/>
+      <c r="B19" s="14"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="14"/>
+      <c r="F19" s="14"/>
+      <c r="G19" s="14"/>
+      <c r="H19" s="14"/>
+      <c r="M19">
+        <v>300</v>
+      </c>
+      <c r="N19">
+        <v>312.7</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" ht="16" customHeight="1">
+      <c r="A20" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="B20" s="9"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="13" t="e">
+        <f>IF($D$17=1,MAX(0.2,MIN(0.75,D10/D9)),NA())</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E20" s="13"/>
+      <c r="F20" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="M20">
+        <v>350</v>
+      </c>
+      <c r="N20">
+        <v>344.4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" ht="16" customHeight="1">
+      <c r="A21" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="B21" s="9"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="13" t="e">
+        <f>IF($D$17=1,(D11/3600)/(PI()*(D9/1000)^2/4),NA())</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E21" s="13"/>
+      <c r="F21" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="M21">
+        <v>400</v>
+      </c>
+      <c r="N21">
+        <v>393.8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" ht="16" customHeight="1">
+      <c r="A22" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="B22" s="9"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="13" t="e">
+        <f>IF($D$17=1,D12*D21*(D9/1000)/(D13/1000),NA())</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E22" s="13"/>
+      <c r="F22" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="M22">
+        <v>500</v>
+      </c>
+      <c r="N22">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" ht="16" customHeight="1">
+      <c r="A23" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="B23" s="9"/>
+      <c r="C23" s="9"/>
+      <c r="D23" s="13" t="e">
+        <f>IF($D$17=1,(SQRT(1-D20^4*(1-D14^2))/(D14*D20^2)-1)^2,NA())</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E23" s="13"/>
+      <c r="F23" s="9" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" ht="16" customHeight="1">
+      <c r="A24" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="B24" s="9"/>
+      <c r="C24" s="9"/>
+      <c r="D24" s="13" t="e">
+        <f>IF($D$17=1,(1-D20^4)/(D14^2*D20^4)*D12*D21^2/200000,NA())</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E24" s="13"/>
+      <c r="F24" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" ht="16" customHeight="1">
+      <c r="A25" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="B25" s="9"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="13" t="e">
+        <f>IF($D$17=1,D23*D12*D21^2/200000,NA())</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E25" s="13"/>
+      <c r="F25" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" ht="16" customHeight="1">
+      <c r="A26" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="B26" s="9"/>
+      <c r="C26" s="9"/>
+      <c r="D26" s="13" t="e">
+        <f>IF($D$17=1,(D11/3600)/(PI()*(D10/1000)^2/4),NA())</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E26" s="13"/>
+      <c r="F26" s="9" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" ht="16" customHeight="1">
+      <c r="A28" s="11" t="s">
+        <v>129</v>
+      </c>
+      <c r="B28" s="11"/>
+      <c r="C28" s="11"/>
+      <c r="D28" s="11"/>
+      <c r="E28" s="11"/>
+      <c r="F28" s="11"/>
+      <c r="G28" s="11"/>
+      <c r="H28" s="11"/>
+    </row>
+    <row r="29" spans="1:14" ht="22" customHeight="1">
+      <c r="A29" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="B29" s="15"/>
+      <c r="C29" s="15"/>
+      <c r="D29" s="15"/>
+      <c r="E29" s="15"/>
+      <c r="F29" s="15"/>
+      <c r="G29" s="15"/>
+      <c r="H29" s="15"/>
+    </row>
+    <row r="30" spans="1:14" ht="22" customHeight="1">
+      <c r="A30" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="B30" s="15"/>
+      <c r="C30" s="15"/>
+      <c r="D30" s="15"/>
+      <c r="E30" s="15"/>
+      <c r="F30" s="15"/>
+      <c r="G30" s="15"/>
+      <c r="H30" s="15"/>
+    </row>
+    <row r="31" spans="1:14" ht="22" customHeight="1">
+      <c r="A31" s="15" t="s">
+        <v>132</v>
+      </c>
+      <c r="B31" s="15"/>
+      <c r="C31" s="15"/>
+      <c r="D31" s="15"/>
+      <c r="E31" s="15"/>
+      <c r="F31" s="15"/>
+      <c r="G31" s="15"/>
+      <c r="H31" s="15"/>
+    </row>
+    <row r="32" spans="1:14" ht="22" customHeight="1">
+      <c r="A32" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="B32" s="15"/>
+      <c r="C32" s="15"/>
+      <c r="D32" s="15"/>
+      <c r="E32" s="15"/>
+      <c r="F32" s="15"/>
+      <c r="G32" s="15"/>
+      <c r="H32" s="15"/>
+    </row>
+    <row r="33" spans="1:8" ht="22" customHeight="1">
+      <c r="A33" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="B33" s="15"/>
+      <c r="C33" s="15"/>
+      <c r="D33" s="15"/>
+      <c r="E33" s="15"/>
+      <c r="F33" s="15"/>
+      <c r="G33" s="15"/>
+      <c r="H33" s="15"/>
+    </row>
+    <row r="34" spans="1:8" ht="22" customHeight="1">
+      <c r="A34" s="15" t="s">
+        <v>135</v>
+      </c>
+      <c r="B34" s="15"/>
+      <c r="C34" s="15"/>
+      <c r="D34" s="15"/>
+      <c r="E34" s="15"/>
+      <c r="F34" s="15"/>
+      <c r="G34" s="15"/>
+      <c r="H34" s="15"/>
+    </row>
+    <row r="36" spans="1:8" ht="16" customHeight="1">
+      <c r="A36" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="B36" s="11"/>
+      <c r="C36" s="11"/>
+      <c r="D36" s="11"/>
+      <c r="E36" s="11"/>
+      <c r="F36" s="11"/>
+      <c r="G36" s="11"/>
+      <c r="H36" s="11"/>
+    </row>
+    <row r="37" spans="1:8" ht="16" customHeight="1">
+      <c r="A37" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="B37" s="9"/>
+      <c r="C37" s="9"/>
+      <c r="D37" s="9"/>
+      <c r="E37" s="9"/>
+      <c r="F37" s="9"/>
+      <c r="G37" s="9"/>
+      <c r="H37" s="9"/>
+    </row>
+    <row r="38" spans="1:8" ht="16" customHeight="1">
+      <c r="A38" s="9"/>
+      <c r="B38" s="9"/>
+      <c r="C38" s="9"/>
+      <c r="D38" s="9"/>
+      <c r="E38" s="9"/>
+      <c r="F38" s="9"/>
+      <c r="G38" s="9"/>
+      <c r="H38" s="9"/>
+    </row>
+    <row r="39" spans="1:8" ht="16" customHeight="1">
+      <c r="A39" s="9"/>
+      <c r="B39" s="9"/>
+      <c r="C39" s="9"/>
+      <c r="D39" s="9"/>
+      <c r="E39" s="9"/>
+      <c r="F39" s="9"/>
+      <c r="G39" s="9"/>
+      <c r="H39" s="9"/>
+    </row>
+    <row r="40" spans="1:8" ht="16" customHeight="1">
+      <c r="A40" s="9"/>
+      <c r="B40" s="9"/>
+      <c r="C40" s="9"/>
+      <c r="D40" s="9"/>
+      <c r="E40" s="9"/>
+      <c r="F40" s="9"/>
+      <c r="G40" s="9"/>
+      <c r="H40" s="9"/>
+    </row>
+    <row r="41" spans="1:8" ht="16" customHeight="1">
+      <c r="A41" s="9"/>
+      <c r="B41" s="9"/>
+      <c r="C41" s="9"/>
+      <c r="D41" s="9"/>
+      <c r="E41" s="9"/>
+      <c r="F41" s="9"/>
+      <c r="G41" s="9"/>
+      <c r="H41" s="9"/>
+    </row>
+    <row r="43" spans="1:8" ht="16" customHeight="1">
+      <c r="A43" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="B43" s="14"/>
+      <c r="C43" s="14"/>
+      <c r="D43" s="14"/>
+      <c r="E43" s="14"/>
+      <c r="F43" s="14"/>
+      <c r="G43" s="14"/>
+      <c r="H43" s="14"/>
+    </row>
+    <row r="44" spans="1:8" ht="16" customHeight="1">
+      <c r="A44" s="14"/>
+      <c r="B44" s="14"/>
+      <c r="C44" s="14"/>
+      <c r="D44" s="14"/>
+      <c r="E44" s="14"/>
+      <c r="F44" s="14"/>
+      <c r="G44" s="14"/>
+      <c r="H44" s="14"/>
+    </row>
+    <row r="45" spans="1:8" ht="16" customHeight="1">
+      <c r="A45" s="14"/>
+      <c r="B45" s="14"/>
+      <c r="C45" s="14"/>
+      <c r="D45" s="14"/>
+      <c r="E45" s="14"/>
+      <c r="F45" s="14"/>
+      <c r="G45" s="14"/>
+      <c r="H45" s="14"/>
+    </row>
+    <row r="47" spans="1:8" ht="16" customHeight="1">
+      <c r="A47" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="B47" s="9"/>
+      <c r="C47" s="9"/>
+      <c r="D47" s="9"/>
+      <c r="E47" s="9"/>
+      <c r="F47" s="9"/>
+      <c r="G47" s="9"/>
+      <c r="H47" s="9"/>
+    </row>
+    <row r="48" spans="1:8" ht="16" customHeight="1">
+      <c r="A48" s="9"/>
+      <c r="B48" s="9"/>
+      <c r="C48" s="9"/>
+      <c r="D48" s="9"/>
+      <c r="E48" s="9"/>
+      <c r="F48" s="9"/>
+      <c r="G48" s="9"/>
+      <c r="H48" s="9"/>
+    </row>
+  </sheetData>
+  <mergeCells count="53">
+    <mergeCell ref="A1:H2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="G10:H15"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="A18:H19"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="A29:H29"/>
+    <mergeCell ref="A30:H30"/>
+    <mergeCell ref="A31:H31"/>
+    <mergeCell ref="A32:H32"/>
+    <mergeCell ref="A33:H33"/>
+    <mergeCell ref="A34:H34"/>
+    <mergeCell ref="A36:H36"/>
+    <mergeCell ref="A37:H41"/>
+    <mergeCell ref="A43:H45"/>
+    <mergeCell ref="A47:H48"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D8">
+      <formula1>$M$5:$M$22</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.3" right="0.3" top="0.35" bottom="0.35" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;BDruckverlust | Engineering&amp;B</oddHeader>
+    <oddFooter>&amp;L&amp;D&amp;RSeite &amp;P von &amp;N</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:U46"/>
+  <sheetFormatPr defaultRowHeight="16" customHeight="1"/>
+  <cols>
+    <col min="1" max="8" width="11.7109375" customWidth="1"/>
+    <col min="14" max="21" width="15.7109375" hidden="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="16" customHeight="1">
+      <c r="A1" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+    </row>
+    <row r="2" spans="1:8" ht="16" customHeight="1">
+      <c r="A2" s="8"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
+    </row>
+    <row r="3" spans="1:8" ht="16" customHeight="1">
+      <c r="A3" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="F3" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
+    </row>
+    <row r="4" spans="1:8" ht="16" customHeight="1">
+      <c r="A4" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="B4" s="10"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="F4" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="G4" s="10"/>
+      <c r="H4" s="10"/>
+    </row>
+    <row r="5" spans="1:8" ht="16" customHeight="1">
+      <c r="A5" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="16" customHeight="1">
+      <c r="A6" s="14" t="s">
+        <v>142</v>
+      </c>
+      <c r="B6" s="14"/>
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
+    </row>
+    <row r="7" spans="1:8" ht="16" customHeight="1">
+      <c r="A7" s="14"/>
+      <c r="B7" s="14"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
+    </row>
+    <row r="8" spans="1:8" ht="16" customHeight="1">
+      <c r="A8" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="9"/>
+    </row>
+    <row r="9" spans="1:8" ht="16" customHeight="1">
+      <c r="A9" s="9"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="9"/>
+    </row>
+    <row r="10" spans="1:8" ht="16" customHeight="1">
+      <c r="A10" s="9"/>
+      <c r="B10" s="9"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+      <c r="H10" s="9"/>
+    </row>
+    <row r="11" spans="1:8" ht="16" customHeight="1">
+      <c r="A11" s="14" t="s">
+        <v>144</v>
+      </c>
+      <c r="B11" s="14"/>
+      <c r="C11" s="14"/>
+      <c r="D11" s="14"/>
+      <c r="E11" s="14"/>
+      <c r="F11" s="14"/>
+      <c r="G11" s="14"/>
+      <c r="H11" s="14"/>
+    </row>
+    <row r="12" spans="1:8" ht="16" customHeight="1">
+      <c r="A12" s="14"/>
+      <c r="B12" s="14"/>
+      <c r="C12" s="14"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="14"/>
+      <c r="F12" s="14"/>
+      <c r="G12" s="14"/>
+      <c r="H12" s="14"/>
+    </row>
+    <row r="13" spans="1:8" ht="16" customHeight="1">
+      <c r="A13" s="14"/>
+      <c r="B13" s="14"/>
+      <c r="C13" s="14"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="14"/>
+      <c r="F13" s="14"/>
+      <c r="G13" s="14"/>
+      <c r="H13" s="14"/>
+    </row>
+    <row r="30" spans="1:8" ht="16" customHeight="1">
+      <c r="A30" s="11" t="s">
+        <v>145</v>
+      </c>
+      <c r="B30" s="11"/>
+      <c r="C30" s="11"/>
+      <c r="D30" s="11"/>
+      <c r="E30" s="11"/>
+      <c r="F30" s="11"/>
+      <c r="G30" s="11"/>
+      <c r="H30" s="11"/>
+    </row>
+    <row r="31" spans="1:8" ht="22" customHeight="1">
+      <c r="A31" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="B31" s="15"/>
+      <c r="C31" s="15"/>
+      <c r="D31" s="15"/>
+      <c r="E31" s="15"/>
+      <c r="F31" s="15"/>
+      <c r="G31" s="15"/>
+      <c r="H31" s="15"/>
+    </row>
+    <row r="32" spans="1:8" ht="22" customHeight="1">
+      <c r="A32" s="15" t="s">
+        <v>147</v>
+      </c>
+      <c r="B32" s="15"/>
+      <c r="C32" s="15"/>
+      <c r="D32" s="15"/>
+      <c r="E32" s="15"/>
+      <c r="F32" s="15"/>
+      <c r="G32" s="15"/>
+      <c r="H32" s="15"/>
+    </row>
+    <row r="33" spans="1:8" ht="22" customHeight="1">
+      <c r="A33" s="15" t="s">
+        <v>148</v>
+      </c>
+      <c r="B33" s="15"/>
+      <c r="C33" s="15"/>
+      <c r="D33" s="15"/>
+      <c r="E33" s="15"/>
+      <c r="F33" s="15"/>
+      <c r="G33" s="15"/>
+      <c r="H33" s="15"/>
+    </row>
+    <row r="34" spans="1:8" ht="22" customHeight="1">
+      <c r="A34" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="B34" s="15"/>
+      <c r="C34" s="15"/>
+      <c r="D34" s="15"/>
+      <c r="E34" s="15"/>
+      <c r="F34" s="15"/>
+      <c r="G34" s="15"/>
+      <c r="H34" s="15"/>
+    </row>
+    <row r="35" spans="1:8" ht="22" customHeight="1">
+      <c r="A35" s="15" t="s">
+        <v>150</v>
+      </c>
+      <c r="B35" s="15"/>
+      <c r="C35" s="15"/>
+      <c r="D35" s="15"/>
+      <c r="E35" s="15"/>
+      <c r="F35" s="15"/>
+      <c r="G35" s="15"/>
+      <c r="H35" s="15"/>
+    </row>
+    <row r="36" spans="1:8" ht="22" customHeight="1">
+      <c r="A36" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="B36" s="15"/>
+      <c r="C36" s="15"/>
+      <c r="D36" s="15"/>
+      <c r="E36" s="15"/>
+      <c r="F36" s="15"/>
+      <c r="G36" s="15"/>
+      <c r="H36" s="15"/>
+    </row>
+    <row r="38" spans="1:8" ht="16" customHeight="1">
+      <c r="A38" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="B38" s="9"/>
+      <c r="C38" s="9"/>
+      <c r="D38" s="9"/>
+      <c r="E38" s="9"/>
+      <c r="F38" s="9"/>
+      <c r="G38" s="9"/>
+      <c r="H38" s="9"/>
+    </row>
+    <row r="39" spans="1:8" ht="16" customHeight="1">
+      <c r="A39" s="9"/>
+      <c r="B39" s="9"/>
+      <c r="C39" s="9"/>
+      <c r="D39" s="9"/>
+      <c r="E39" s="9"/>
+      <c r="F39" s="9"/>
+      <c r="G39" s="9"/>
+      <c r="H39" s="9"/>
+    </row>
+    <row r="40" spans="1:8" ht="16" customHeight="1">
+      <c r="A40" s="9"/>
+      <c r="B40" s="9"/>
+      <c r="C40" s="9"/>
+      <c r="D40" s="9"/>
+      <c r="E40" s="9"/>
+      <c r="F40" s="9"/>
+      <c r="G40" s="9"/>
+      <c r="H40" s="9"/>
+    </row>
+    <row r="41" spans="1:8" ht="16" customHeight="1">
+      <c r="A41" s="9"/>
+      <c r="B41" s="9"/>
+      <c r="C41" s="9"/>
+      <c r="D41" s="9"/>
+      <c r="E41" s="9"/>
+      <c r="F41" s="9"/>
+      <c r="G41" s="9"/>
+      <c r="H41" s="9"/>
+    </row>
+    <row r="43" spans="1:8" ht="16" customHeight="1">
+      <c r="A43" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="B43" s="9"/>
+      <c r="C43" s="9"/>
+      <c r="D43" s="9"/>
+      <c r="E43" s="9"/>
+      <c r="F43" s="9"/>
+      <c r="G43" s="9"/>
+      <c r="H43" s="9"/>
+    </row>
+    <row r="44" spans="1:8" ht="16" customHeight="1">
+      <c r="A44" s="9"/>
+      <c r="B44" s="9"/>
+      <c r="C44" s="9"/>
+      <c r="D44" s="9"/>
+      <c r="E44" s="9"/>
+      <c r="F44" s="9"/>
+      <c r="G44" s="9"/>
+      <c r="H44" s="9"/>
+    </row>
+    <row r="46" spans="1:8" ht="16" customHeight="1">
+      <c r="A46" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="B46" s="11"/>
+      <c r="C46" s="11"/>
+      <c r="D46" s="11"/>
+      <c r="E46" s="11"/>
+      <c r="F46" s="11"/>
+      <c r="G46" s="11"/>
+      <c r="H46" s="11"/>
+    </row>
+  </sheetData>
+  <mergeCells count="19">
+    <mergeCell ref="A1:H2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A6:H7"/>
+    <mergeCell ref="A8:H10"/>
+    <mergeCell ref="A11:H13"/>
+    <mergeCell ref="A30:H30"/>
+    <mergeCell ref="A31:H31"/>
+    <mergeCell ref="A32:H32"/>
+    <mergeCell ref="A33:H33"/>
+    <mergeCell ref="A34:H34"/>
+    <mergeCell ref="A35:H35"/>
+    <mergeCell ref="A36:H36"/>
+    <mergeCell ref="A38:H41"/>
+    <mergeCell ref="A43:H44"/>
+    <mergeCell ref="A46:H46"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D5">
+      <formula1>0</formula1>
+      <formula2>1</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.3" right="0.3" top="0.35" bottom="0.35" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="95" orientation="portrait"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;BDruckverlust | Engineering&amp;B</oddHeader>
+    <oddFooter>&amp;L&amp;D&amp;RSeite &amp;P von &amp;N</oddFooter>
+  </headerFooter>
+  <rowBreaks count="1" manualBreakCount="1">
+    <brk id="44" max="16383" man="1"/>
+  </rowBreaks>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add standalone printable Kv pressure drop workbook and integrated sheet
</commit_message>
<xml_diff>
--- a/excel/Druckverlust_Vorlage.xlsx
+++ b/excel/Druckverlust_Vorlage.xlsx
@@ -16,11 +16,13 @@
     <sheet name="KvArmatur" sheetId="7" r:id="rId7"/>
     <sheet name="Blende_Standalone" sheetId="8" r:id="rId8"/>
     <sheet name="Systembericht" sheetId="9" r:id="rId9"/>
+    <sheet name="Kv_Standalone" sheetId="10" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="ArmaturenTypen">'Armaturendatenbank'!$A$5:$A$16</definedName>
     <definedName name="DNWerte">'Armaturendatenbank'!$F$5:$F$22</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="7">Blende_Standalone!$A$1:$H$48</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="9">Kv_Standalone!$A$1:$H$48</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="8">Systembericht!$A$1:$H$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -74,7 +76,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="175">
   <si>
     <t>Rohrleitungs-Systemkennlinie</t>
   </si>
@@ -539,6 +541,66 @@
   </si>
   <si>
     <t>ANHANG | vollstaendiger Berechnungsstand</t>
+  </si>
+  <si>
+    <t>Kv-Armatur | Druckverlustberechnung</t>
+  </si>
+  <si>
+    <t>EINGABEN | unabhaengig von der Systemberechnung</t>
+  </si>
+  <si>
+    <t>Kv bei aktueller Oeffnung</t>
+  </si>
+  <si>
+    <t>Dyn. Viskositaet (dokumentiert)</t>
+  </si>
+  <si>
+    <t>Kv fuer die gewaehlte Oeffnung aus Herstellerdaten einsetzen. Kvs gilt nur bei voller Oeffnung. Anzahl gilt fuer gleiche Armaturen in Serie, nicht parallel.</t>
+  </si>
+  <si>
+    <t>Druckverlust je Armatur</t>
+  </si>
+  <si>
+    <t>Gesamtdruckverlust in Serie</t>
+  </si>
+  <si>
+    <t>Gesamtdruckverlust</t>
+  </si>
+  <si>
+    <t>Pa</t>
+  </si>
+  <si>
+    <t>Verlusthoehe der Fluessigkeit</t>
+  </si>
+  <si>
+    <t>BERECHNUNGSFORMELN | Kv-Definition</t>
+  </si>
+  <si>
+    <t>ρref = 1000 kg/m³; Kv: Volumenstrom bei Δp = 1 bar fuer Referenzwasser</t>
+  </si>
+  <si>
+    <t>Δpeinzeln [bar] = (ρ/ρref) · (Q/Kv)²</t>
+  </si>
+  <si>
+    <t>Δpgesamt [bar] = n · Δpeinzeln [bar]</t>
+  </si>
+  <si>
+    <t>Δp [Pa] = 100000 · Δp [bar]</t>
+  </si>
+  <si>
+    <t>hVerlust [m] = Δpgesamt [Pa] / (ρ g); g = 9,80665 m/s²</t>
+  </si>
+  <si>
+    <t>Q und Kv in m³/h; ρ in kg/m³; bei Q = 0 gilt Δp = 0</t>
+  </si>
+  <si>
+    <t>Stationaere, einphasige inkompressible Newtonsche Fluessigkeit; konstante Dichte und Armaturenoeffnung. Einfache Kv-Beziehung fuer turbulente, nicht kavitierende Stroemung. Keine Korrektur fuer Viskositaet, Reynolds-Zahl, FL, Kavitation, Flashing oder Choked Flow. Viskositaet und Temperatur sind nur dokumentiert. Kein Rohr-/Blendenmodell; DN und Lochdurchmesser gehoeren zur separaten Blendenberechnung. Kv-Definition im Kontext IEC 60534-2-1, keine vollstaendige normgerechte Regelventilauslegung.</t>
+  </si>
+  <si>
+    <t>Ohne Makros und ohne Verknuepfungen zu anderen Blaettern. Ergebnisse aktualisieren sich mit Excel-Formeln. Fuer Engineering-Freigabe Kv, Stoffwerte und Anwendungsgrenzen pruefen. A4 Hochformat, eine Seite.</t>
+  </si>
+  <si>
+    <t>Geprueft durch: ____________________  Datum: ____________  Freigabe: ______________</t>
   </si>
 </sst>
 </file>
@@ -684,7 +746,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -713,6 +775,8 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1935,6 +1999,563 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:H48"/>
+  <sheetFormatPr defaultRowHeight="16" customHeight="1"/>
+  <cols>
+    <col min="1" max="8" width="11.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="16" customHeight="1">
+      <c r="A1" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+    </row>
+    <row r="2" spans="1:8" ht="16" customHeight="1">
+      <c r="A2" s="8"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
+    </row>
+    <row r="3" spans="1:8" ht="16" customHeight="1">
+      <c r="A3" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="B3" s="16"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="F3" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="G3" s="16"/>
+      <c r="H3" s="16"/>
+    </row>
+    <row r="4" spans="1:8" ht="16" customHeight="1">
+      <c r="A4" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="B4" s="16"/>
+      <c r="C4" s="16"/>
+      <c r="D4" s="16"/>
+      <c r="F4" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="G4" s="16"/>
+      <c r="H4" s="16"/>
+    </row>
+    <row r="6" spans="1:8" ht="16" customHeight="1">
+      <c r="A6" s="11" t="s">
+        <v>156</v>
+      </c>
+      <c r="B6" s="11"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="11"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+    </row>
+    <row r="8" spans="1:8" ht="16" customHeight="1">
+      <c r="A8" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="17">
+        <v>10</v>
+      </c>
+      <c r="E8" s="17"/>
+      <c r="F8" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="G8" s="14" t="s">
+        <v>159</v>
+      </c>
+      <c r="H8" s="14"/>
+    </row>
+    <row r="9" spans="1:8" ht="16" customHeight="1">
+      <c r="A9" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="B9" s="9"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="17">
+        <v>10</v>
+      </c>
+      <c r="E9" s="17"/>
+      <c r="F9" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="G9" s="14"/>
+      <c r="H9" s="14"/>
+    </row>
+    <row r="10" spans="1:8" ht="16" customHeight="1">
+      <c r="A10" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="B10" s="9"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="17">
+        <v>1000</v>
+      </c>
+      <c r="E10" s="17"/>
+      <c r="F10" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="G10" s="14"/>
+      <c r="H10" s="14"/>
+    </row>
+    <row r="11" spans="1:8" ht="16" customHeight="1">
+      <c r="A11" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="B11" s="9"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="17">
+        <v>1</v>
+      </c>
+      <c r="E11" s="17"/>
+      <c r="F11" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="G11" s="14"/>
+      <c r="H11" s="14"/>
+    </row>
+    <row r="12" spans="1:8" ht="16" customHeight="1">
+      <c r="A12" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="17">
+        <v>1</v>
+      </c>
+      <c r="E12" s="17"/>
+      <c r="F12" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G12" s="14"/>
+      <c r="H12" s="14"/>
+    </row>
+    <row r="13" spans="1:8" ht="16" customHeight="1">
+      <c r="A13" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="17">
+        <v>20</v>
+      </c>
+      <c r="E13" s="17"/>
+      <c r="F13" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="G13" s="14"/>
+      <c r="H13" s="14"/>
+    </row>
+    <row r="16" spans="1:8" ht="16" customHeight="1">
+      <c r="A16" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="13">
+        <f>IFERROR(IF(AND(ISNUMBER(D8),ISNUMBER(D9),ISNUMBER(D10),ISNUMBER(D11),ISNUMBER(D12),D8&gt;=0,D9&gt;0,D10&gt;0,D11&gt;=1,D11&lt;=1000,D11=INT(D11),D12&gt;0,OR(ISBLANK(D13),AND(ISNUMBER(D13),D13&gt;=-273.15))),1,0),0)</f>
+        <v>0</v>
+      </c>
+      <c r="E16" s="13"/>
+    </row>
+    <row r="17" spans="1:8" ht="16" customHeight="1">
+      <c r="A17" s="14" t="str">
+        <f>IF(D16&lt;&gt;1,"UNGUELTIG: Eingaben pruefen; Ergebnisse nicht verwendbar.","Kv-Naeherung: turbulent, konstante Oeffnung, nicht kavitierend. Herstellergrenzen pruefen; keine Viskositaetskorrektur.")</f>
+        <v>Beim Oeffnen in Excel neu berechnen.</v>
+      </c>
+      <c r="B17" s="14"/>
+      <c r="C17" s="14"/>
+      <c r="D17" s="14"/>
+      <c r="E17" s="14"/>
+      <c r="F17" s="14"/>
+      <c r="G17" s="14"/>
+      <c r="H17" s="14"/>
+    </row>
+    <row r="18" spans="1:8" ht="16" customHeight="1">
+      <c r="A18" s="14"/>
+      <c r="B18" s="14"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="14"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="14"/>
+      <c r="H18" s="14"/>
+    </row>
+    <row r="19" spans="1:8" ht="16" customHeight="1">
+      <c r="A19" s="14"/>
+      <c r="B19" s="14"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="14"/>
+      <c r="F19" s="14"/>
+      <c r="G19" s="14"/>
+      <c r="H19" s="14"/>
+    </row>
+    <row r="21" spans="1:8" ht="16" customHeight="1">
+      <c r="A21" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="B21" s="9"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="13" t="e">
+        <f>IF($D$16=1,(D10/1000)*(D8/D9)^2,NA())</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E21" s="13"/>
+      <c r="F21" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="16" customHeight="1">
+      <c r="A22" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="B22" s="9"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="13" t="e">
+        <f>IF($D$16=1,D11*(D10/1000)*(D8/D9)^2,NA())</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E22" s="13"/>
+      <c r="F22" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="16" customHeight="1">
+      <c r="A23" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="B23" s="9"/>
+      <c r="C23" s="9"/>
+      <c r="D23" s="13" t="e">
+        <f>IF($D$16=1,D22*100000,NA())</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E23" s="13"/>
+      <c r="F23" s="9" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="16" customHeight="1">
+      <c r="A24" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="B24" s="9"/>
+      <c r="C24" s="9"/>
+      <c r="D24" s="13" t="e">
+        <f>IF($D$16=1,D22*100000/(D10*9.80665),NA())</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E24" s="13"/>
+      <c r="F24" s="9" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="16" customHeight="1">
+      <c r="A27" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="B27" s="11"/>
+      <c r="C27" s="11"/>
+      <c r="D27" s="11"/>
+      <c r="E27" s="11"/>
+      <c r="F27" s="11"/>
+      <c r="G27" s="11"/>
+      <c r="H27" s="11"/>
+    </row>
+    <row r="28" spans="1:8" ht="22" customHeight="1">
+      <c r="A28" s="15" t="s">
+        <v>166</v>
+      </c>
+      <c r="B28" s="15"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="15"/>
+      <c r="F28" s="15"/>
+      <c r="G28" s="15"/>
+      <c r="H28" s="15"/>
+    </row>
+    <row r="29" spans="1:8" ht="22" customHeight="1">
+      <c r="A29" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="B29" s="15"/>
+      <c r="C29" s="15"/>
+      <c r="D29" s="15"/>
+      <c r="E29" s="15"/>
+      <c r="F29" s="15"/>
+      <c r="G29" s="15"/>
+      <c r="H29" s="15"/>
+    </row>
+    <row r="30" spans="1:8" ht="22" customHeight="1">
+      <c r="A30" s="15" t="s">
+        <v>168</v>
+      </c>
+      <c r="B30" s="15"/>
+      <c r="C30" s="15"/>
+      <c r="D30" s="15"/>
+      <c r="E30" s="15"/>
+      <c r="F30" s="15"/>
+      <c r="G30" s="15"/>
+      <c r="H30" s="15"/>
+    </row>
+    <row r="31" spans="1:8" ht="22" customHeight="1">
+      <c r="A31" s="15" t="s">
+        <v>169</v>
+      </c>
+      <c r="B31" s="15"/>
+      <c r="C31" s="15"/>
+      <c r="D31" s="15"/>
+      <c r="E31" s="15"/>
+      <c r="F31" s="15"/>
+      <c r="G31" s="15"/>
+      <c r="H31" s="15"/>
+    </row>
+    <row r="32" spans="1:8" ht="22" customHeight="1">
+      <c r="A32" s="15" t="s">
+        <v>170</v>
+      </c>
+      <c r="B32" s="15"/>
+      <c r="C32" s="15"/>
+      <c r="D32" s="15"/>
+      <c r="E32" s="15"/>
+      <c r="F32" s="15"/>
+      <c r="G32" s="15"/>
+      <c r="H32" s="15"/>
+    </row>
+    <row r="33" spans="1:8" ht="22" customHeight="1">
+      <c r="A33" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="B33" s="15"/>
+      <c r="C33" s="15"/>
+      <c r="D33" s="15"/>
+      <c r="E33" s="15"/>
+      <c r="F33" s="15"/>
+      <c r="G33" s="15"/>
+      <c r="H33" s="15"/>
+    </row>
+    <row r="35" spans="1:8" ht="16" customHeight="1">
+      <c r="A35" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="B35" s="11"/>
+      <c r="C35" s="11"/>
+      <c r="D35" s="11"/>
+      <c r="E35" s="11"/>
+      <c r="F35" s="11"/>
+      <c r="G35" s="11"/>
+      <c r="H35" s="11"/>
+    </row>
+    <row r="36" spans="1:8" ht="16" customHeight="1">
+      <c r="A36" s="9" t="s">
+        <v>172</v>
+      </c>
+      <c r="B36" s="9"/>
+      <c r="C36" s="9"/>
+      <c r="D36" s="9"/>
+      <c r="E36" s="9"/>
+      <c r="F36" s="9"/>
+      <c r="G36" s="9"/>
+      <c r="H36" s="9"/>
+    </row>
+    <row r="37" spans="1:8" ht="16" customHeight="1">
+      <c r="A37" s="9"/>
+      <c r="B37" s="9"/>
+      <c r="C37" s="9"/>
+      <c r="D37" s="9"/>
+      <c r="E37" s="9"/>
+      <c r="F37" s="9"/>
+      <c r="G37" s="9"/>
+      <c r="H37" s="9"/>
+    </row>
+    <row r="38" spans="1:8" ht="16" customHeight="1">
+      <c r="A38" s="9"/>
+      <c r="B38" s="9"/>
+      <c r="C38" s="9"/>
+      <c r="D38" s="9"/>
+      <c r="E38" s="9"/>
+      <c r="F38" s="9"/>
+      <c r="G38" s="9"/>
+      <c r="H38" s="9"/>
+    </row>
+    <row r="39" spans="1:8" ht="16" customHeight="1">
+      <c r="A39" s="9"/>
+      <c r="B39" s="9"/>
+      <c r="C39" s="9"/>
+      <c r="D39" s="9"/>
+      <c r="E39" s="9"/>
+      <c r="F39" s="9"/>
+      <c r="G39" s="9"/>
+      <c r="H39" s="9"/>
+    </row>
+    <row r="40" spans="1:8" ht="16" customHeight="1">
+      <c r="A40" s="9"/>
+      <c r="B40" s="9"/>
+      <c r="C40" s="9"/>
+      <c r="D40" s="9"/>
+      <c r="E40" s="9"/>
+      <c r="F40" s="9"/>
+      <c r="G40" s="9"/>
+      <c r="H40" s="9"/>
+    </row>
+    <row r="41" spans="1:8" ht="16" customHeight="1">
+      <c r="A41" s="9"/>
+      <c r="B41" s="9"/>
+      <c r="C41" s="9"/>
+      <c r="D41" s="9"/>
+      <c r="E41" s="9"/>
+      <c r="F41" s="9"/>
+      <c r="G41" s="9"/>
+      <c r="H41" s="9"/>
+    </row>
+    <row r="43" spans="1:8" ht="16" customHeight="1">
+      <c r="A43" s="14" t="s">
+        <v>173</v>
+      </c>
+      <c r="B43" s="14"/>
+      <c r="C43" s="14"/>
+      <c r="D43" s="14"/>
+      <c r="E43" s="14"/>
+      <c r="F43" s="14"/>
+      <c r="G43" s="14"/>
+      <c r="H43" s="14"/>
+    </row>
+    <row r="44" spans="1:8" ht="16" customHeight="1">
+      <c r="A44" s="14"/>
+      <c r="B44" s="14"/>
+      <c r="C44" s="14"/>
+      <c r="D44" s="14"/>
+      <c r="E44" s="14"/>
+      <c r="F44" s="14"/>
+      <c r="G44" s="14"/>
+      <c r="H44" s="14"/>
+    </row>
+    <row r="45" spans="1:8" ht="16" customHeight="1">
+      <c r="A45" s="14"/>
+      <c r="B45" s="14"/>
+      <c r="C45" s="14"/>
+      <c r="D45" s="14"/>
+      <c r="E45" s="14"/>
+      <c r="F45" s="14"/>
+      <c r="G45" s="14"/>
+      <c r="H45" s="14"/>
+    </row>
+    <row r="47" spans="1:8" ht="16" customHeight="1">
+      <c r="A47" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="B47" s="9"/>
+      <c r="C47" s="9"/>
+      <c r="D47" s="9"/>
+      <c r="E47" s="9"/>
+      <c r="F47" s="9"/>
+      <c r="G47" s="9"/>
+      <c r="H47" s="9"/>
+    </row>
+    <row r="48" spans="1:8" ht="16" customHeight="1">
+      <c r="A48" s="9"/>
+      <c r="B48" s="9"/>
+      <c r="C48" s="9"/>
+      <c r="D48" s="9"/>
+      <c r="E48" s="9"/>
+      <c r="F48" s="9"/>
+      <c r="G48" s="9"/>
+      <c r="H48" s="9"/>
+    </row>
+  </sheetData>
+  <mergeCells count="41">
+    <mergeCell ref="A1:H2"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="G8:H13"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="A17:H19"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="A27:H27"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="A29:H29"/>
+    <mergeCell ref="A30:H30"/>
+    <mergeCell ref="A31:H31"/>
+    <mergeCell ref="A32:H32"/>
+    <mergeCell ref="A33:H33"/>
+    <mergeCell ref="A35:H35"/>
+    <mergeCell ref="A36:H41"/>
+    <mergeCell ref="A43:H45"/>
+    <mergeCell ref="A47:H48"/>
+  </mergeCells>
+  <dataValidations count="5">
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D9">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D10">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D12">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D8">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D11">
+      <formula1>1</formula1>
+      <formula2>1000</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.3" right="0.3" top="0.35" bottom="0.35" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
+  <headerFooter>
+    <oddHeader>&amp;C&amp;BDruckverlust | Engineering&amp;B</oddHeader>
+    <oddFooter>&amp;L&amp;D&amp;RSeite &amp;P von &amp;N</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M4"/>

</xml_diff>